<commit_message>
Plantilla gratuita: titulo a ancho completo + instrucciones de como abrirla en Google Sheets
</commit_message>
<xml_diff>
--- a/descarga-gratuita/Control-Notas-2026-2027.xlsx
+++ b/descarga-gratuita/Control-Notas-2026-2027.xlsx
@@ -50,7 +50,12 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="17"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -72,11 +77,6 @@
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="10"/>
     </font>
     <font>
       <i val="1"/>
@@ -133,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -150,6 +150,9 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -168,22 +171,22 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -628,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -705,33 +708,68 @@
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>DIFERENCIA CON LA VERSIÓN DE PAGO</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="76" customHeight="1">
+          <t>CÓMO ABRIRLO (si no tienes Excel, sin problema)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="25" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Este archivo gratuito solo controla NOTAS. El Organizador de Estudios 2026-2027 completo (calculafacil.app/organizador-estudios/) además incluye: asistencia día a día con semáforo verde/ámbar/rojo, registro de faltas, retrasos y justificadas, tabla por asignatura automática y tu cuadro de mandos con objetivo de nota.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>LICENCIA</t>
+          <t>1. Con Microsoft Excel (Windows/Mac): doble clic en el archivo y listo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="59" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2. Sin Excel, con Google Sheets (gratis y sin instalar): entra en drive.google.com → Nuevo → Subir archivo → elige este archivo .xlsx → doble clic sobre el archivo subido y se abrirá solo en Google Sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>3. O instala LibreOffice (gratis): tras instalarlo, doble clic en el archivo y se abre igual.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>¿Solo te ofrece el Bloc de notas? Botón derecho sobre el archivo → Abrir con → elige Excel, Google Sheets o LibreOffice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>DIFERENCIA CON LA VERSIÓN DE PAGO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="76" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Este archivo gratuito solo controla NOTAS. El Organizador de Estudios 2026-2027 completo (calculafacil.app/organizador-estudios/) además incluye: asistencia día a día con semáforo verde/ámbar/rojo, registro de faltas, retrasos y justificadas, tabla por asignatura automática y tu cuadro de mandos con objetivo de nota.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>LICENCIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="42" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
           <t>Puedes usar esta versión gratuita libremente para tu curso. No la revendas ni la subas a portales de pago.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="24" ht="25" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>CalculaFácil · calculafacil.app · plantilla para estudiantes</t>
         </is>
@@ -739,21 +777,26 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="0" insertHyperlinks="0" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="0" insertColumns="0" pivotTables="0" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
-  <mergeCells count="14">
+  <mergeCells count="19">
+    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A20:F20"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A8:F8"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToWidth="1"/>
@@ -767,7 +810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:I23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -782,264 +825,271 @@
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="B1" s="5" t="inlineStr">
+    <row r="1" ht="46" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>CONTROL RÁPIDO DE NOTAS 2026/2027</t>
         </is>
       </c>
     </row>
     <row r="2" ht="23" customHeight="1">
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Hasta 5 notas por asignatura · PESO (%) · la NOTA FINAL se calcula sola</t>
         </is>
       </c>
     </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>CALCULAFÁCIL · calculafacil.app · versión gratuita</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>ASIGNATURA</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>NOTA 1</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>NOTA 2</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>NOTA 3</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>NOTA 4</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>NOTA 5</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>PESO (%)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="9">
+      <c r="B5" s="8" t="inlineStr"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="10">
         <f>IF($B5="","",ROUND(AVERAGE(C5:G5),2))</f>
         <v/>
       </c>
-      <c r="I5" s="10" t="n"/>
+      <c r="I5" s="11" t="n"/>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="9">
+      <c r="B6" s="8" t="inlineStr"/>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="10">
         <f>IF($B6="","",ROUND(AVERAGE(C6:G6),2))</f>
         <v/>
       </c>
-      <c r="I6" s="10" t="n"/>
+      <c r="I6" s="11" t="n"/>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="9">
+      <c r="B7" s="8" t="inlineStr"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="10">
         <f>IF($B7="","",ROUND(AVERAGE(C7:G7),2))</f>
         <v/>
       </c>
-      <c r="I7" s="10" t="n"/>
+      <c r="I7" s="11" t="n"/>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="B8" s="7" t="inlineStr"/>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="9">
+      <c r="B8" s="8" t="inlineStr"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="10">
         <f>IF($B8="","",ROUND(AVERAGE(C8:G8),2))</f>
         <v/>
       </c>
-      <c r="I8" s="10" t="n"/>
+      <c r="I8" s="11" t="n"/>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="B9" s="7" t="inlineStr"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
-      <c r="H9" s="9">
+      <c r="B9" s="8" t="inlineStr"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="10">
         <f>IF($B9="","",ROUND(AVERAGE(C9:G9),2))</f>
         <v/>
       </c>
-      <c r="I9" s="10" t="n"/>
+      <c r="I9" s="11" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="7" t="inlineStr"/>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="9">
+      <c r="B10" s="8" t="inlineStr"/>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="10">
         <f>IF($B10="","",ROUND(AVERAGE(C10:G10),2))</f>
         <v/>
       </c>
-      <c r="I10" s="10" t="n"/>
+      <c r="I10" s="11" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="B11" s="7" t="inlineStr"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="9">
+      <c r="B11" s="8" t="inlineStr"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="10">
         <f>IF($B11="","",ROUND(AVERAGE(C11:G11),2))</f>
         <v/>
       </c>
-      <c r="I11" s="10" t="n"/>
+      <c r="I11" s="11" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="B12" s="7" t="inlineStr"/>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
-      <c r="H12" s="9">
+      <c r="B12" s="8" t="inlineStr"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="10">
         <f>IF($B12="","",ROUND(AVERAGE(C12:G12),2))</f>
         <v/>
       </c>
-      <c r="I12" s="10" t="n"/>
+      <c r="I12" s="11" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="B13" s="7" t="inlineStr"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
-      <c r="H13" s="9">
+      <c r="B13" s="8" t="inlineStr"/>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="10">
         <f>IF($B13="","",ROUND(AVERAGE(C13:G13),2))</f>
         <v/>
       </c>
-      <c r="I13" s="10" t="n"/>
+      <c r="I13" s="11" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="B14" s="7" t="inlineStr"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="8" t="n"/>
-      <c r="G14" s="8" t="n"/>
-      <c r="H14" s="9">
+      <c r="B14" s="8" t="inlineStr"/>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="9" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="10">
         <f>IF($B14="","",ROUND(AVERAGE(C14:G14),2))</f>
         <v/>
       </c>
-      <c r="I14" s="10" t="n"/>
+      <c r="I14" s="11" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="B15" s="7" t="inlineStr"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="8" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="8" t="n"/>
-      <c r="G15" s="8" t="n"/>
-      <c r="H15" s="9">
+      <c r="B15" s="8" t="inlineStr"/>
+      <c r="C15" s="9" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="10">
         <f>IF($B15="","",ROUND(AVERAGE(C15:G15),2))</f>
         <v/>
       </c>
-      <c r="I15" s="10" t="n"/>
+      <c r="I15" s="11" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="B16" s="7" t="inlineStr"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="8" t="n"/>
-      <c r="G16" s="8" t="n"/>
-      <c r="H16" s="9">
+      <c r="B16" s="8" t="inlineStr"/>
+      <c r="C16" s="9" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="10">
         <f>IF($B16="","",ROUND(AVERAGE(C16:G16),2))</f>
         <v/>
       </c>
-      <c r="I16" s="10" t="n"/>
+      <c r="I16" s="11" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1"/>
     <row r="18" ht="26" customHeight="1">
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>RESUMEN</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>TOTAL PESO (%)</t>
         </is>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="14">
         <f>SUM(I5:I16)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>NOTA FINAL PONDERADA</t>
         </is>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="15">
         <f>IF(C19=0,"",ROUND(SUMPRODUCT(N(H5:H16),I5:I16)/C19,2))</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="40" customHeight="1">
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>La NOTA FINAL PONDERADA usa los pesos de tu centro. Solo cuentan las asignaturas con nota. Si tu centro pondera de otra forma, ajusta los PESO (%) hasta que el TOTAL sume 100 y se ponga verde.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>¿Quieres también el control de FALTAS y el cuadro de mandos? Mira el Organizador de Estudios completo en calculafacil.app/organizador-estudios/</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="17" t="inlineStr">
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>CalculaFácil · calculafacil.app · versión gratuita</t>
         </is>
@@ -1047,13 +1097,14 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="0" insertHyperlinks="0" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="0" insertColumns="0" pivotTables="0" deleteRows="0" formatCells="0" formatRows="0" sort="0" password="CF7C"/>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="B22:I22"/>
+    <mergeCell ref="A3:I3"/>
     <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:H16">
     <cfRule type="expression" priority="1" dxfId="0">

</xml_diff>